<commit_message>
Fix IPO float parsing
</commit_message>
<xml_diff>
--- a/ipo_watch_results.xlsx
+++ b/ipo_watch_results.xlsx
@@ -1102,10 +1102,18 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>26.76%</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>유</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
@@ -1398,7 +1406,7 @@
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>76.55%</t>
+          <t>21.12%</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>

</xml_diff>

<commit_message>
Fix IPO market caps
</commit_message>
<xml_diff>
--- a/ipo_watch_results.xlsx
+++ b/ipo_watch_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W21"/>
+  <dimension ref="A1:W20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,7 +584,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -593,37 +593,79 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>기도산업</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>봉제의복 제조업</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>미래에셋증권, 삼성증권</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>213.31</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>32.41%</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>66.92%</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1664억</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>유</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>28400</v>
+      </c>
+      <c r="P3" t="n">
+        <v>28000</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>-1.41%</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>18580</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>-33.64%</t>
+        </is>
+      </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
@@ -631,7 +673,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -640,79 +682,59 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>기도산업</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>봉제의복 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>미래에셋증권, 삼성증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>213.31</v>
+        <v>219.56</v>
       </c>
       <c r="H4" t="n">
-        <v>5.63</v>
+        <v>1047.78</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
+          <t>8.98%</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>66.92%</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>66.92%</t>
-        </is>
-      </c>
+          <t>28.61%</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>1660억</t>
+          <t>1222억</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>유</t>
+          <t>무</t>
         </is>
       </c>
       <c r="O4" t="n">
-        <v>28400</v>
-      </c>
-      <c r="P4" t="n">
-        <v>28000</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>-1.41%</t>
-        </is>
-      </c>
-      <c r="R4" t="n">
-        <v>18580</v>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>-33.64%</t>
-        </is>
-      </c>
+        <v>10000</v>
+      </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
@@ -720,7 +742,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -729,7 +751,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>니어스랩</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -739,35 +761,43 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>219.56</v>
+        <v>743.49</v>
       </c>
       <c r="H5" t="n">
-        <v>1047.78</v>
+        <v>529.99</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>8.98%</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
+          <t>1.26%</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>39.42%</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>28.66%</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
+          <t>37.15%</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>32.49%</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>1222억</t>
+          <t>2380억</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -776,12 +806,24 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>10000</v>
-      </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
+        <v>41200</v>
+      </c>
+      <c r="P5" t="n">
+        <v>40500</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>-1.70%</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>28650</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>-29.26%</t>
+        </is>
+      </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
@@ -789,7 +831,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -798,53 +840,43 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>니어스랩</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>항공기,우주선 및 부품 제조업</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>743.49</v>
-      </c>
-      <c r="H6" t="n">
-        <v>529.99</v>
-      </c>
+        <v>868.64</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1.26%</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>39.42%</t>
-        </is>
-      </c>
+          <t>4.05%</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>37.19%</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>32.49%</t>
-        </is>
-      </c>
+          <t>40.11%</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2380억</t>
+          <t>2759억</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -853,24 +885,12 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>41200</v>
-      </c>
-      <c r="P6" t="n">
-        <v>40500</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>-1.70%</t>
-        </is>
-      </c>
-      <c r="R6" t="n">
-        <v>28650</v>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>-29.26%</t>
-        </is>
-      </c>
+        <v>14600</v>
+      </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
@@ -878,7 +898,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -887,57 +907,79 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>딜리셔스</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>항공기,우주선 및 부품 제조업</t>
+          <t>무점포 소매업</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>868.64</v>
-      </c>
-      <c r="H7" t="inlineStr"/>
+        <v>184.06</v>
+      </c>
+      <c r="H7" t="n">
+        <v>10.29</v>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>4.05%</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
+          <t>0.10%</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>6.24%</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>40.15%</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
+          <t>36.89%</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>36.42%</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2000억</t>
+          <t>1532억</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>유</t>
         </is>
       </c>
       <c r="O7" t="n">
-        <v>14600</v>
-      </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
+        <v>7000</v>
+      </c>
+      <c r="P7" t="n">
+        <v>6000</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>-14.29%</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>5140</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>-14.33%</t>
+        </is>
+      </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
@@ -945,7 +987,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -954,43 +996,53 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>항공기,우주선 및 부품 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>KB증권</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>868.64</v>
-      </c>
-      <c r="H8" t="inlineStr"/>
+        <v>1146.41</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1706.71</v>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4.05%</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
+          <t>17.93%</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>77.50%</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>40.15%</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
+          <t>41.03%</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>31.89%</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2000억</t>
+          <t>1579억</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -999,20 +1051,44 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>14600</v>
-      </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
+        <v>20700</v>
+      </c>
+      <c r="P8" t="n">
+        <v>30750</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>48.55%</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>22000</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>-28.46%</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>31000.0</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>49.76%</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>51190.0</t>
+        </is>
+      </c>
       <c r="W8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1021,87 +1097,99 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>딜리셔스</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>무점포 소매업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>KB증권</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>184.06</v>
+        <v>1238</v>
       </c>
       <c r="H9" t="n">
-        <v>10.29</v>
+        <v>1510.57</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0.10%</t>
+          <t>6.92%</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>6.24%</t>
+          <t>74.17%</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>36.93%</t>
+          <t>33.19%</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>36.42%</t>
+          <t>24.86%</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>1532억</t>
+          <t>1335억</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>유</t>
+          <t>무</t>
         </is>
       </c>
       <c r="O9" t="n">
-        <v>7000</v>
+        <v>10000</v>
       </c>
       <c r="P9" t="n">
-        <v>6000</v>
+        <v>16560</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>-14.29%</t>
+          <t>65.60%</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>5140</v>
+        <v>9400</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>-14.33%</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
+          <t>-43.24%</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>18740.0</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>87.40%</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>69621.0</t>
+        </is>
+      </c>
       <c r="W9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1110,99 +1198,55 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>레메디</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>KB증권</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>1146.41</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1706.71</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>17.93%</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>77.50%</t>
-        </is>
-      </c>
+          <t>IBK투자증권</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>41.03%</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>31.89%</t>
-        </is>
-      </c>
+          <t>26.42%</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>1579억</t>
+          <t>1875억</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>유</t>
         </is>
       </c>
       <c r="O10" t="n">
-        <v>20700</v>
-      </c>
-      <c r="P10" t="n">
-        <v>30750</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>48.55%</t>
-        </is>
-      </c>
-      <c r="R10" t="n">
-        <v>22000</v>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>-28.46%</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>31000.0</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>49.76%</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>51190.0</t>
-        </is>
-      </c>
+        <v>16500</v>
+      </c>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1211,7 +1255,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1221,89 +1265,55 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>KB증권</t>
+          <t>유진투자증권, 미래에셋증권</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>1238</v>
-      </c>
-      <c r="H11" t="n">
-        <v>1510.57</v>
-      </c>
+        <v>1109.37</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>6.92%</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>74.17%</t>
-        </is>
-      </c>
+          <t>98.72%</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>33.19%</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>24.86%</t>
-        </is>
-      </c>
+          <t>26.76%</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
-          <t>1335억</t>
+          <t>1849억</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>무</t>
+          <t>유</t>
         </is>
       </c>
       <c r="O11" t="n">
-        <v>10000</v>
-      </c>
-      <c r="P11" t="n">
-        <v>16560</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>65.60%</t>
-        </is>
-      </c>
-      <c r="R11" t="n">
-        <v>9400</v>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>-43.24%</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>18740.0</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>87.40%</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>69621.0</t>
-        </is>
-      </c>
+        <v>18000</v>
+      </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1312,57 +1322,79 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>스카이랩스</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>유진투자증권, 미래에셋증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1109.37</v>
-      </c>
-      <c r="H12" t="inlineStr"/>
+        <v>63.41</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2.85</v>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>98.72%</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
+          <t>0.17%</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>10.93%</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>26.76%</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
+          <t>27.26%</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>26.42%</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>10억</t>
+          <t>1876억</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>유</t>
+          <t>무</t>
         </is>
       </c>
       <c r="O12" t="n">
-        <v>18000</v>
-      </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
+        <v>10000</v>
+      </c>
+      <c r="P12" t="n">
+        <v>8500</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>-15.00%</t>
+        </is>
+      </c>
+      <c r="R12" t="n">
+        <v>23500</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>176.47%</t>
+        </is>
+      </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr"/>
@@ -1370,7 +1402,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1379,53 +1411,53 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>스카이랩스</t>
+          <t>에이치엘지노믹스</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>기초 의약물질 제조업</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>KB증권, IBK투자증권</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>63.41</v>
+        <v>714.52</v>
       </c>
       <c r="H13" t="n">
-        <v>2.85</v>
+        <v>666.78</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>1.91%</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>10.93%</t>
+          <t>34.58%</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>27.29%</t>
+          <t>33.00%</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>26.42%</t>
+          <t>24.41%</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>1876억</t>
+          <t>1673억</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1434,22 +1466,22 @@
         </is>
       </c>
       <c r="O13" t="n">
-        <v>10000</v>
+        <v>21500</v>
       </c>
       <c r="P13" t="n">
-        <v>8500</v>
+        <v>21500</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>-15.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>23500</v>
+        <v>14790</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>176.47%</t>
+          <t>-31.21%</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
@@ -1459,86 +1491,60 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>스펙</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>에이치엘지노믹스</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>기초 의약물질 제조업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>KB증권, IBK투자증권</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>714.52</v>
-      </c>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>666.78</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>1.91%</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>34.58%</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>33.00%</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>24.41%</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>1673억</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>무</t>
-        </is>
-      </c>
+        <v>357</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="n">
-        <v>21500</v>
+        <v>2000</v>
       </c>
       <c r="P14" t="n">
-        <v>21500</v>
+        <v>4000</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="R14" t="n">
-        <v>14790</v>
+        <v>2075</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>-31.21%</t>
+          <t>-48.12%</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -1548,62 +1554,68 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>스펙</t>
+          <t>일반</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>기타 생활용품 소매업</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1248.47</v>
+      </c>
       <c r="H15" t="n">
-        <v>357</v>
-      </c>
-      <c r="I15" t="inlineStr"/>
+        <v>1477.65</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>3.65%</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>21.08%</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>1202억</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
       <c r="O15" t="n">
-        <v>2000</v>
-      </c>
-      <c r="P15" t="n">
-        <v>4000</v>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-      <c r="R15" t="n">
-        <v>2075</v>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>-48.12%</t>
-        </is>
-      </c>
+        <v>12000</v>
+      </c>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
@@ -1611,7 +1623,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1620,45 +1632,53 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>인제니아테라퓨틱스</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>기타 생활용품 소매업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1248.47</v>
+        <v>50.4</v>
       </c>
       <c r="H16" t="n">
-        <v>1477.65</v>
+        <v>3.09</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>3.65%</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr"/>
+          <t>2.23%</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>3.17%</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>21.12%</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
+          <t>25.60%</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>25.36%</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>1200억</t>
+          <t>5933억</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1669,10 +1689,22 @@
       <c r="O16" t="n">
         <v>12000</v>
       </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
+      <c r="P16" t="n">
+        <v>10960</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>-8.67%</t>
+        </is>
+      </c>
+      <c r="R16" t="n">
+        <v>17990</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>64.14%</t>
+        </is>
+      </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
@@ -1680,88 +1712,50 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>스펙</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>인제니아테라퓨틱스</t>
+          <t>케이비제34호스팩</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>KB증권</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>50.4</v>
-      </c>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>3.09</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>2.23%</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>3.17%</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>25.60%</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>25.36%</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>5933억</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>무</t>
-        </is>
-      </c>
+        <v>397.33</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="n">
-        <v>12000</v>
-      </c>
-      <c r="P17" t="n">
-        <v>10960</v>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>-8.67%</t>
-        </is>
-      </c>
-      <c r="R17" t="n">
-        <v>17990</v>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>64.14%</t>
-        </is>
-      </c>
+        <v>2000</v>
+      </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
@@ -1769,296 +1763,245 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>스펙</t>
+          <t>일반</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>케이비제34호스팩</t>
+          <t>케이앤에스아이앤씨</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>통신 및 방송 장비 제조업</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>KB증권</t>
+          <t>IBK투자증권</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>938.24</v>
+      </c>
       <c r="H18" t="n">
-        <v>397.33</v>
-      </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
+        <v>1079.55</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>0.78%</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>71.42%</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>30.03%</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>17.59%</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>1129억</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
       <c r="O18" t="n">
-        <v>2000</v>
-      </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
+        <v>11000</v>
+      </c>
+      <c r="P18" t="n">
+        <v>21000</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>90.91%</t>
+        </is>
+      </c>
+      <c r="R18" t="n">
+        <v>15380</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>-26.76%</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>23450.0</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>113.18%</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>309228.0</t>
+        </is>
+      </c>
       <c r="W18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>스펙</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>케이앤에스아이앤씨</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>통신 및 방송 장비 제조업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>IBK투자증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>938.24</v>
-      </c>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>1079.55</v>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>0.78%</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>71.42%</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>30.00%</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>17.59%</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>1129억</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>무</t>
-        </is>
-      </c>
+        <v>494.62</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="n">
-        <v>11000</v>
-      </c>
-      <c r="P19" t="n">
-        <v>21000</v>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>90.91%</t>
-        </is>
-      </c>
-      <c r="R19" t="n">
-        <v>15380</v>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>-26.76%</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>23450.0</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>113.18%</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>309228.0</t>
-        </is>
-      </c>
+        <v>2000</v>
+      </c>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>스펙</t>
+          <t>일반</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>해치텍</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>DB증권</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>101.91</v>
+      </c>
       <c r="H20" t="n">
-        <v>494.62</v>
-      </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+        <v>25.73</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>15.08%</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>5.63%</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>38.35%</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>37.69%</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>1271억</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
       <c r="O20" t="n">
-        <v>2000</v>
-      </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
+        <v>23000</v>
+      </c>
+      <c r="P20" t="n">
+        <v>20500</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>-10.87%</t>
+        </is>
+      </c>
+      <c r="R20" t="n">
+        <v>13930</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>-32.05%</t>
+        </is>
+      </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
     </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>14</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>일반</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>해치텍</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>반도체 제조업</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>DB증권</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>101.91</v>
-      </c>
-      <c r="H21" t="n">
-        <v>25.73</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>15.08%</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>5.63%</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>38.42%</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>37.69%</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>1269억</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>무</t>
-        </is>
-      </c>
-      <c r="O21" t="n">
-        <v>23000</v>
-      </c>
-      <c r="P21" t="n">
-        <v>20500</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>-10.87%</t>
-        </is>
-      </c>
-      <c r="R21" t="n">
-        <v>13930</v>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>-32.05%</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix DART company matching
</commit_message>
<xml_diff>
--- a/ipo_watch_results.xlsx
+++ b/ipo_watch_results.xlsx
@@ -564,15 +564,35 @@
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>123.19</v>
+      </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.27%</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>22.19%</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>1965억</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>무</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>10000</v>
+      </c>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>

</xml_diff>

<commit_message>
Fix IPO allocation lockup parsing
</commit_message>
<xml_diff>
--- a/ipo_watch_results.xlsx
+++ b/ipo_watch_results.xlsx
@@ -575,13 +575,21 @@
           <t>0.27%</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>33.00%</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>22.19%</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>17.15%</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>1965억</t>
@@ -733,13 +741,21 @@
           <t>8.98%</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>44.02%</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>28.61%</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>23.21%</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr">
         <is>
           <t>1222억</t>
@@ -903,13 +919,21 @@
           <t>4.05%</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>57.26%</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>40.11%</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>33.29%</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr">
         <is>
           <t>2759억</t>
@@ -1263,13 +1287,21 @@
           <t>21.75%</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>85.39%</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>26.42%</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>21.01%</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr">
         <is>
           <t>1875억</t>
@@ -1650,13 +1682,21 @@
           <t>3.65%</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>55.61%</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>21.08%</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>14.42%</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
           <t>1202억</t>

</xml_diff>